<commit_message>
update status change logic from pocket for all modules
</commit_message>
<xml_diff>
--- a/frontend/src/assets/templates/templateForUploadDocumentLines.xlsx
+++ b/frontend/src/assets/templates/templateForUploadDocumentLines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Projects\fullStack\admin-panel-copy\new\scanmate-admin-panel\frontend\src\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8ADD6D-E2D1-4A53-B009-BB09A31AF320}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE33DE6-0EA9-488D-A4D3-95A6FECEE23F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
   <si>
     <t>Id</t>
   </si>
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.85546875" customWidth="1"/>
@@ -803,6 +803,41 @@
         <v>35</v>
       </c>
     </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>